<commit_message>
added latest qualifying results
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B2CE78-33BD-4663-A072-9B31EB1D98AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669C03D1-8FA3-4601-A97D-55A84CECB655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
@@ -12499,7 +12499,9 @@
       <c r="G102" s="8">
         <v>1</v>
       </c>
-      <c r="H102" s="8"/>
+      <c r="H102" s="8">
+        <v>1</v>
+      </c>
       <c r="I102" t="s">
         <v>88</v>
       </c>
@@ -12539,7 +12541,9 @@
       <c r="G103" s="8">
         <v>7</v>
       </c>
-      <c r="H103" s="8"/>
+      <c r="H103" s="8">
+        <v>2</v>
+      </c>
       <c r="I103" t="s">
         <v>88</v>
       </c>
@@ -12579,7 +12583,9 @@
       <c r="G104" s="8">
         <v>2</v>
       </c>
-      <c r="H104" s="8"/>
+      <c r="H104" s="8">
+        <v>3</v>
+      </c>
       <c r="I104" t="s">
         <v>88</v>
       </c>
@@ -12619,7 +12625,9 @@
       <c r="G105" s="8">
         <v>3</v>
       </c>
-      <c r="H105" s="8"/>
+      <c r="H105" s="8">
+        <v>4</v>
+      </c>
       <c r="I105" t="s">
         <v>88</v>
       </c>
@@ -12659,7 +12667,9 @@
       <c r="G106" s="8">
         <v>8</v>
       </c>
-      <c r="H106" s="8"/>
+      <c r="H106" s="8">
+        <v>5</v>
+      </c>
       <c r="I106" t="s">
         <v>88</v>
       </c>
@@ -12699,7 +12709,9 @@
       <c r="G107" s="8">
         <v>9</v>
       </c>
-      <c r="H107" s="8"/>
+      <c r="H107" s="8">
+        <v>6</v>
+      </c>
       <c r="I107" t="s">
         <v>88</v>
       </c>
@@ -12739,7 +12751,9 @@
       <c r="G108" s="8">
         <v>4</v>
       </c>
-      <c r="H108" s="8"/>
+      <c r="H108" s="8">
+        <v>7</v>
+      </c>
       <c r="I108" t="s">
         <v>88</v>
       </c>
@@ -12779,7 +12793,9 @@
       <c r="G109" s="8">
         <v>5</v>
       </c>
-      <c r="H109" s="8"/>
+      <c r="H109" s="8">
+        <v>8</v>
+      </c>
       <c r="I109" t="s">
         <v>88</v>
       </c>
@@ -12819,7 +12835,9 @@
       <c r="G110" s="8">
         <v>10</v>
       </c>
-      <c r="H110" s="8"/>
+      <c r="H110" s="8">
+        <v>9</v>
+      </c>
       <c r="I110" t="s">
         <v>88</v>
       </c>
@@ -12859,7 +12877,9 @@
       <c r="G111" s="8">
         <v>11</v>
       </c>
-      <c r="H111" s="8"/>
+      <c r="H111" s="8">
+        <v>10</v>
+      </c>
       <c r="I111" t="s">
         <v>88</v>
       </c>
@@ -12899,7 +12919,9 @@
       <c r="G112" s="8">
         <v>6</v>
       </c>
-      <c r="H112" s="8"/>
+      <c r="H112" s="8">
+        <v>11</v>
+      </c>
       <c r="I112" t="s">
         <v>88</v>
       </c>
@@ -12939,7 +12961,9 @@
       <c r="G113" s="8">
         <v>13</v>
       </c>
-      <c r="H113" s="8"/>
+      <c r="H113" s="8">
+        <v>12</v>
+      </c>
       <c r="I113" t="s">
         <v>88</v>
       </c>
@@ -12979,7 +13003,9 @@
       <c r="G114" s="8">
         <v>14</v>
       </c>
-      <c r="H114" s="8"/>
+      <c r="H114" s="8">
+        <v>13</v>
+      </c>
       <c r="I114" t="s">
         <v>88</v>
       </c>
@@ -13019,7 +13045,9 @@
       <c r="G115" s="8">
         <v>15</v>
       </c>
-      <c r="H115" s="8"/>
+      <c r="H115" s="8">
+        <v>14</v>
+      </c>
       <c r="I115" t="s">
         <v>88</v>
       </c>
@@ -13059,7 +13087,9 @@
       <c r="G116" s="8">
         <v>16</v>
       </c>
-      <c r="H116" s="8"/>
+      <c r="H116" s="8">
+        <v>15</v>
+      </c>
       <c r="I116" t="s">
         <v>88</v>
       </c>
@@ -13099,7 +13129,9 @@
       <c r="G117" s="8">
         <v>17</v>
       </c>
-      <c r="H117" s="8"/>
+      <c r="H117" s="8">
+        <v>16</v>
+      </c>
       <c r="I117" t="s">
         <v>88</v>
       </c>
@@ -13139,7 +13171,9 @@
       <c r="G118" s="8">
         <v>23</v>
       </c>
-      <c r="H118" s="8"/>
+      <c r="H118" s="8">
+        <v>17</v>
+      </c>
       <c r="I118" t="s">
         <v>88</v>
       </c>
@@ -13179,7 +13213,9 @@
       <c r="G119" s="8">
         <v>18</v>
       </c>
-      <c r="H119" s="8"/>
+      <c r="H119" s="8">
+        <v>18</v>
+      </c>
       <c r="I119" t="s">
         <v>88</v>
       </c>
@@ -13219,7 +13255,9 @@
       <c r="G120" s="8">
         <v>19</v>
       </c>
-      <c r="H120" s="8"/>
+      <c r="H120" s="8">
+        <v>19</v>
+      </c>
       <c r="I120" t="s">
         <v>88</v>
       </c>
@@ -13259,7 +13297,9 @@
       <c r="G121" s="8">
         <v>20</v>
       </c>
-      <c r="H121" s="8"/>
+      <c r="H121" s="8">
+        <v>20</v>
+      </c>
       <c r="I121" t="s">
         <v>88</v>
       </c>
@@ -13299,7 +13339,9 @@
       <c r="G122" s="8">
         <v>21</v>
       </c>
-      <c r="H122" s="8"/>
+      <c r="H122" s="8">
+        <v>21</v>
+      </c>
       <c r="I122" t="s">
         <v>88</v>
       </c>
@@ -13339,7 +13381,9 @@
       <c r="G123" s="8">
         <v>12</v>
       </c>
-      <c r="H123" s="8"/>
+      <c r="H123" s="8">
+        <v>22</v>
+      </c>
       <c r="I123" t="s">
         <v>88</v>
       </c>
@@ -13379,7 +13423,9 @@
       <c r="G124" s="8">
         <v>22</v>
       </c>
-      <c r="H124" s="8"/>
+      <c r="H124" s="8">
+        <v>23</v>
+      </c>
       <c r="I124" t="s">
         <v>88</v>
       </c>
@@ -13419,7 +13465,9 @@
       <c r="G125" s="8">
         <v>24</v>
       </c>
-      <c r="H125" s="8"/>
+      <c r="H125" s="8">
+        <v>24</v>
+      </c>
       <c r="I125" t="s">
         <v>88</v>
       </c>
@@ -13459,7 +13507,9 @@
       <c r="G126" s="8">
         <v>25</v>
       </c>
-      <c r="H126" s="8"/>
+      <c r="H126" s="8">
+        <v>25</v>
+      </c>
       <c r="I126" t="s">
         <v>88</v>
       </c>

</xml_diff>

<commit_message>
Moved IndyCar files to IndyCar/ folder
</commit_message>
<xml_diff>
--- a/IndyCar/predictions/model_compare.xlsx
+++ b/IndyCar/predictions/model_compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\IndyCar\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669C03D1-8FA3-4601-A97D-55A84CECB655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79064C1-D40F-499D-8B73-BC87BDB142F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="3" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
@@ -6611,7 +6611,9 @@
       <c r="G102" s="8">
         <v>1</v>
       </c>
-      <c r="H102" s="8"/>
+      <c r="H102" s="8">
+        <v>1</v>
+      </c>
       <c r="I102" t="s">
         <v>88</v>
       </c>
@@ -6651,7 +6653,9 @@
       <c r="G103" s="8">
         <v>7</v>
       </c>
-      <c r="H103" s="8"/>
+      <c r="H103" s="8">
+        <v>3</v>
+      </c>
       <c r="I103" t="s">
         <v>88</v>
       </c>
@@ -6691,7 +6695,9 @@
       <c r="G104" s="8">
         <v>2</v>
       </c>
-      <c r="H104" s="8"/>
+      <c r="H104" s="8">
+        <v>4</v>
+      </c>
       <c r="I104" t="s">
         <v>88</v>
       </c>
@@ -6731,7 +6737,9 @@
       <c r="G105" s="8">
         <v>8</v>
       </c>
-      <c r="H105" s="8"/>
+      <c r="H105" s="8">
+        <v>6</v>
+      </c>
       <c r="I105" t="s">
         <v>88</v>
       </c>
@@ -6771,7 +6779,9 @@
       <c r="G106" s="8">
         <v>9</v>
       </c>
-      <c r="H106" s="8"/>
+      <c r="H106" s="8">
+        <v>14</v>
+      </c>
       <c r="I106" t="s">
         <v>88</v>
       </c>
@@ -6811,7 +6821,9 @@
       <c r="G107" s="8">
         <v>3</v>
       </c>
-      <c r="H107" s="8"/>
+      <c r="H107" s="8">
+        <v>5</v>
+      </c>
       <c r="I107" t="s">
         <v>88</v>
       </c>
@@ -6851,7 +6863,9 @@
       <c r="G108" s="8">
         <v>4</v>
       </c>
-      <c r="H108" s="8"/>
+      <c r="H108" s="8">
+        <v>20</v>
+      </c>
       <c r="I108" t="s">
         <v>88</v>
       </c>
@@ -6891,7 +6905,9 @@
       <c r="G109" s="8">
         <v>11</v>
       </c>
-      <c r="H109" s="8"/>
+      <c r="H109" s="8">
+        <v>24</v>
+      </c>
       <c r="I109" t="s">
         <v>88</v>
       </c>
@@ -6931,7 +6947,9 @@
       <c r="G110" s="8">
         <v>5</v>
       </c>
-      <c r="H110" s="8"/>
+      <c r="H110" s="8">
+        <v>19</v>
+      </c>
       <c r="I110" t="s">
         <v>88</v>
       </c>
@@ -6971,7 +6989,9 @@
       <c r="G111" s="8">
         <v>6</v>
       </c>
-      <c r="H111" s="8"/>
+      <c r="H111" s="8">
+        <v>7</v>
+      </c>
       <c r="I111" t="s">
         <v>88</v>
       </c>
@@ -7011,7 +7031,9 @@
       <c r="G112" s="8">
         <v>12</v>
       </c>
-      <c r="H112" s="8"/>
+      <c r="H112" s="8">
+        <v>25</v>
+      </c>
       <c r="I112" t="s">
         <v>88</v>
       </c>
@@ -7051,7 +7073,9 @@
       <c r="G113" s="8">
         <v>13</v>
       </c>
-      <c r="H113" s="8"/>
+      <c r="H113" s="8">
+        <v>9</v>
+      </c>
       <c r="I113" t="s">
         <v>88</v>
       </c>
@@ -7091,7 +7115,9 @@
       <c r="G114" s="8">
         <v>14</v>
       </c>
-      <c r="H114" s="8"/>
+      <c r="H114" s="8">
+        <v>10</v>
+      </c>
       <c r="I114" t="s">
         <v>88</v>
       </c>
@@ -7131,7 +7157,9 @@
       <c r="G115" s="8">
         <v>15</v>
       </c>
-      <c r="H115" s="8"/>
+      <c r="H115" s="8">
+        <v>2</v>
+      </c>
       <c r="I115" t="s">
         <v>88</v>
       </c>
@@ -7171,7 +7199,9 @@
       <c r="G116" s="8">
         <v>16</v>
       </c>
-      <c r="H116" s="8"/>
+      <c r="H116" s="8">
+        <v>8</v>
+      </c>
       <c r="I116" t="s">
         <v>88</v>
       </c>
@@ -7211,7 +7241,9 @@
       <c r="G117" s="8">
         <v>17</v>
       </c>
-      <c r="H117" s="8"/>
+      <c r="H117" s="8">
+        <v>11</v>
+      </c>
       <c r="I117" t="s">
         <v>88</v>
       </c>
@@ -7251,7 +7283,9 @@
       <c r="G118" s="8">
         <v>18</v>
       </c>
-      <c r="H118" s="8"/>
+      <c r="H118" s="8">
+        <v>13</v>
+      </c>
       <c r="I118" t="s">
         <v>88</v>
       </c>
@@ -7291,7 +7325,9 @@
       <c r="G119" s="8">
         <v>23</v>
       </c>
-      <c r="H119" s="8"/>
+      <c r="H119" s="8">
+        <v>15</v>
+      </c>
       <c r="I119" t="s">
         <v>88</v>
       </c>
@@ -7331,7 +7367,9 @@
       <c r="G120" s="8">
         <v>19</v>
       </c>
-      <c r="H120" s="8"/>
+      <c r="H120" s="8">
+        <v>18</v>
+      </c>
       <c r="I120" t="s">
         <v>88</v>
       </c>
@@ -7371,7 +7409,9 @@
       <c r="G121" s="8">
         <v>10</v>
       </c>
-      <c r="H121" s="8"/>
+      <c r="H121" s="8">
+        <v>21</v>
+      </c>
       <c r="I121" t="s">
         <v>88</v>
       </c>
@@ -7411,7 +7451,9 @@
       <c r="G122" s="8">
         <v>20</v>
       </c>
-      <c r="H122" s="8"/>
+      <c r="H122" s="8">
+        <v>16</v>
+      </c>
       <c r="I122" t="s">
         <v>88</v>
       </c>
@@ -7451,7 +7493,9 @@
       <c r="G123" s="8">
         <v>21</v>
       </c>
-      <c r="H123" s="8"/>
+      <c r="H123" s="8">
+        <v>22</v>
+      </c>
       <c r="I123" t="s">
         <v>88</v>
       </c>
@@ -7491,7 +7535,9 @@
       <c r="G124" s="8">
         <v>24</v>
       </c>
-      <c r="H124" s="8"/>
+      <c r="H124" s="8">
+        <v>12</v>
+      </c>
       <c r="I124" t="s">
         <v>88</v>
       </c>
@@ -7531,7 +7577,9 @@
       <c r="G125" s="8">
         <v>22</v>
       </c>
-      <c r="H125" s="8"/>
+      <c r="H125" s="8">
+        <v>17</v>
+      </c>
       <c r="I125" t="s">
         <v>88</v>
       </c>
@@ -7571,7 +7619,9 @@
       <c r="G126" s="8">
         <v>25</v>
       </c>
-      <c r="H126" s="8"/>
+      <c r="H126" s="8">
+        <v>23</v>
+      </c>
       <c r="I126" t="s">
         <v>88</v>
       </c>
@@ -12542,7 +12592,7 @@
         <v>7</v>
       </c>
       <c r="H103" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I103" t="s">
         <v>88</v>
@@ -12584,7 +12634,7 @@
         <v>2</v>
       </c>
       <c r="H104" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I104" t="s">
         <v>88</v>
@@ -12626,7 +12676,7 @@
         <v>3</v>
       </c>
       <c r="H105" s="8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I105" t="s">
         <v>88</v>
@@ -12668,7 +12718,7 @@
         <v>8</v>
       </c>
       <c r="H106" s="8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I106" t="s">
         <v>88</v>
@@ -12710,7 +12760,7 @@
         <v>9</v>
       </c>
       <c r="H107" s="8">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="I107" t="s">
         <v>88</v>
@@ -12752,7 +12802,7 @@
         <v>4</v>
       </c>
       <c r="H108" s="8">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I108" t="s">
         <v>88</v>
@@ -12794,7 +12844,7 @@
         <v>5</v>
       </c>
       <c r="H109" s="8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I109" t="s">
         <v>88</v>
@@ -12836,7 +12886,7 @@
         <v>10</v>
       </c>
       <c r="H110" s="8">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I110" t="s">
         <v>88</v>
@@ -12920,7 +12970,7 @@
         <v>6</v>
       </c>
       <c r="H112" s="8">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="I112" t="s">
         <v>88</v>
@@ -12962,7 +13012,7 @@
         <v>13</v>
       </c>
       <c r="H113" s="8">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="I113" t="s">
         <v>88</v>
@@ -13004,7 +13054,7 @@
         <v>14</v>
       </c>
       <c r="H114" s="8">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I114" t="s">
         <v>88</v>
@@ -13046,7 +13096,7 @@
         <v>15</v>
       </c>
       <c r="H115" s="8">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="I115" t="s">
         <v>88</v>
@@ -13088,7 +13138,7 @@
         <v>16</v>
       </c>
       <c r="H116" s="8">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="I116" t="s">
         <v>88</v>
@@ -13130,7 +13180,7 @@
         <v>17</v>
       </c>
       <c r="H117" s="8">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="I117" t="s">
         <v>88</v>
@@ -13172,7 +13222,7 @@
         <v>23</v>
       </c>
       <c r="H118" s="8">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I118" t="s">
         <v>88</v>
@@ -13214,7 +13264,7 @@
         <v>18</v>
       </c>
       <c r="H119" s="8">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I119" t="s">
         <v>88</v>
@@ -13256,7 +13306,7 @@
         <v>19</v>
       </c>
       <c r="H120" s="8">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I120" t="s">
         <v>88</v>
@@ -13298,7 +13348,7 @@
         <v>20</v>
       </c>
       <c r="H121" s="8">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I121" t="s">
         <v>88</v>
@@ -13340,7 +13390,7 @@
         <v>21</v>
       </c>
       <c r="H122" s="8">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I122" t="s">
         <v>88</v>
@@ -13382,7 +13432,7 @@
         <v>12</v>
       </c>
       <c r="H123" s="8">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I123" t="s">
         <v>88</v>
@@ -13424,7 +13474,7 @@
         <v>22</v>
       </c>
       <c r="H124" s="8">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I124" t="s">
         <v>88</v>
@@ -13466,7 +13516,7 @@
         <v>24</v>
       </c>
       <c r="H125" s="8">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="I125" t="s">
         <v>88</v>
@@ -13508,7 +13558,7 @@
         <v>25</v>
       </c>
       <c r="H126" s="8">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I126" t="s">
         <v>88</v>

</xml_diff>